<commit_message>
feat: expandir catalogo para 29 obras, logo no header, GA4 e dados estruturados completos
- Adiciona simbolo do brasao a esquerda do nome no header (mobile-first)
- Amplia catalogo de 12 para 29 obras com capas, links de afiliado e sinopses
- Atualiza links de afiliado e sinopses das 12 obras originais
- Sincroniza JSON-LD (structured data) com as sinopses atuais para as 29 obras
- Instala Google Analytics (gtag.js) no head
</commit_message>
<xml_diff>
--- a/keywords-seo-domenico-falco.xlsx
+++ b/keywords-seo-domenico-falco.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b1c62caea10bc3cc/BackUp/2. Carreira/1. JF Design/Projetos/Livros Dô/Site/livrosdofalco/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_CA952BE50894C943AE6235916204CD1F85A3ED23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9DC4A70-EA77-4046-BD3C-80573188BF5D}"/>
+  <xr:revisionPtr revIDLastSave="130" documentId="11_CA952BE50894C943AE6235916204CD1F85A3ED23" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4C4272A-AFAA-44A8-865C-9D1276F1FAC0}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="860" windowWidth="21330" windowHeight="11540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pilares SEO" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="202">
   <si>
     <t>Keywords por Pilar — Domenico Falco</t>
   </si>
@@ -406,13 +406,240 @@
   </si>
   <si>
     <t>URL Loja Amazon</t>
+  </si>
+  <si>
+    <t>Destinos Cruzados</t>
+  </si>
+  <si>
+    <t>Um Lugar ao Sol</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0hDr3Z3s</t>
+  </si>
+  <si>
+    <t>O livro conta a trajetória de tres jovens amigos, uma inglesa, um chines e um indiano, durante as decadas de 1940/50, e como os principais fatos históricos dessa época, suas crenças e decisões afetaram suas vidas.</t>
+  </si>
+  <si>
+    <t>Sinopse</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0aGQgpeB</t>
+  </si>
+  <si>
+    <t>O livro conta a história de cinco alunos de um institudo de artes cenicas em Nova Iorque nos anos 1960 e 1970, os quais são envolvidos nas grandes transformações culturais daquelas decadas, incluindo a guerra do Vietnã.</t>
+  </si>
+  <si>
+    <t>O livro conta a historia de um jovem ingles do século XIX apaixonado por aventuras e desejoso de conhecer o mundo.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B03lGhsxT</t>
+  </si>
+  <si>
+    <t>O Siciliano</t>
+  </si>
+  <si>
+    <t>O livro conta a historia de Matteo, um siciliano que se vê obrigado a migrar para o Brasil, devido as consequencias da disputa de terras na região em que vivia com sua familia. Sua tragetoria como imigrante acontece nas primeiras décadas do século XX e se desenvolve nas cidades do Rio de Janero e São Paulo.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B08t0ClRq</t>
+  </si>
+  <si>
+    <t>James, o jovem explorador inglês, que estava desaparecido havia muitos meses, finalmente foi encontrado em seu navio o qual estava a deriva proximo à costa da Antártida, por uma embarcação de pesquisa da Argentina . Após seu resgate e, devido ao seu péssimo estado de saúde e do trauma que haiva sofrido no mar, James ficou sem memória. Durante o período de recuperação, ele recebeu a atenção e os cuidados de Luna, uma cientista da tripulação argentina. Depois de se recuparar , ambos descobrem que compartilham da mesma paixão pela exploração do planeta. Assim, juntos passam por grandes aventuras em Galápagos e na Amazônia Andina em busca do desconhecido.</t>
+  </si>
+  <si>
+    <t>O Explorador - Em busca do desconhecido</t>
+  </si>
+  <si>
+    <t>O Tesouro Maldito</t>
+  </si>
+  <si>
+    <t>No início do século XVI, o capitão Diego Garcia e seus marinheiros roubam um grande tesouro dos Astecas, mas são amaldiçoados por um alto sacerdote durante a fuga da cidade de Tenochtitlán. Enquanto navegam pelos mares do Caribe em busca de refugio, misteriosos eventos atormentam a tripulação, culminando com a presença de uma terrível criatura a bordo.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B079khqVa</t>
+  </si>
+  <si>
+    <t>A Teia</t>
+  </si>
+  <si>
+    <t>Joca e Helena são dois jovens nascidos em favelas do Rio de Janeiro. Idealista, ela queria estudar para ajudar a familia e viver em segurança, além de auxiliar tambem os mais necessitados.
+Ele queria ser jogador de futebol, como a grande maioria dos meninos da comunidade, para ficar rico e famoso.
+Mais tarde, já adultos, seus caminhos se cruzam.
+Joca é um criminoso, dono de empresas e muito rico. Ela é promotora publica e tem como missão desbaratar um grande esquema de lavagem de dinheiro do tráfego e de sites de apostas ilegais, onde o alvo é justamente o império de Joca..
+O choque de princípios é inevitável, mas nada dura para sempre, em um meio com tantas controversias.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B06lJ8s2p</t>
+  </si>
+  <si>
+    <t>Trata-se de um drama vivido por Kilian e Eileen, dois jovens de Belfast na Irlanda do Norte, que se apaixonam e constituem familia durante os anos duros dos conflitos entre católicos e protestantes nas décadas de 60 e 70, principalmente.
+Amor, tradição, religião , injustiça, vingança e o acaso, afetam de maneira dramática a vida da pequena familia, influenciando em suas escolhas e os destinos de cada um deles</t>
+  </si>
+  <si>
+    <t>O que eu lembro deles</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B03B5r7zc</t>
+  </si>
+  <si>
+    <t>A Viagem</t>
+  </si>
+  <si>
+    <t>O livro conta o drama vivido por três casais de jovens ricos em uma viagem pelo Mediterrâneo a bordo yate de luxo "Aurora". O confinamento e os acontecimentos imprevisíveis colocam em cheque suas crenças e emoções, afetando tragicamente o destino deles e da tripulação.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0gD3RC5M</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B08KUy5xA</t>
+  </si>
+  <si>
+    <t>o Asilo</t>
+  </si>
+  <si>
+    <t>O livro explora o relacionamento dos idosos, em sua maioria enfermos, que vivem no Asilo Sao Pedro no município de Bela Vista, próximo a cidade do Rio de Janeiro, em meados do século XX.</t>
+  </si>
+  <si>
+    <t>A indústria do vício</t>
+  </si>
+  <si>
+    <t>O romance se passa durante a época da Lei Seca (1920 -1933) nas cidades de Nova Iorque, Nova Jersey e Atlantic City, com mais de 10 personagens sendo Don Domenico o capo da máfia e Vince seu conselheiro, que se aproveitam financeiramente desse difícil período da história norte americana.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B09juTmUd</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B08IDAJBy</t>
+  </si>
+  <si>
+    <t>O livro conta a história da irreverente Joana, de seus familiares, amores e aventuras, durante a primeira metade do século XX na França e no Brasil.</t>
+  </si>
+  <si>
+    <t>O livro conta as aventuras de um casal de portugueses, para implantar engenhos e explorar as riquezas geradas pela cana de açúcar no Brasil colonial do século XVI .</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0eEyJ9Zy</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B01k8LazN</t>
+  </si>
+  <si>
+    <t>as aventuras de um corsário inglês que se torna pirata durante o século XVIII, percorrendo os principais oceanos da terra.</t>
+  </si>
+  <si>
+    <t>O livro conta história de uma família de italianos que busca melhores condições de vida na America do norte e do Sul, Trata-se de uma ficção baseada em alguns fatos reais, que se desenrola durante todo o século XX e início do século XXI , retratando os principais eventos históricos ocorridos neste período.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0a17JfGu</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B01MYHAbP</t>
+  </si>
+  <si>
+    <t>Reflexões sobre a vida</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0b0XZSET</t>
+  </si>
+  <si>
+    <t>Reflexões e pensamentos sobre vida de forma geral e também sobre a pandemia .</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B05HgVbe9</t>
+  </si>
+  <si>
+    <t>uma família que, apesar de sofrer uma grande injustiça, consegue se reerguer aproveitando as oportunidades que a vida lhes ofereceu de modo inesperado. O romance ficcional se passa no Japão feudal.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0fxnejMl</t>
+  </si>
+  <si>
+    <t>dois cavaleiros templários e suas aventuras na Terra Santa e na Europa, em busca do Santo Graal.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0bjfPAhK</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0gm2f63E</t>
+  </si>
+  <si>
+    <t>um romano que nasceu na mesma época de Jesus (Yeshua), tendo sua vida afetada pelo legado dele.</t>
+  </si>
+  <si>
+    <t>o sofrimento e os esforços de um homem, escravisado desde seu nascimento, para vencer o preconceito e o ódio, motivados pela sua condição humana. A história acontece em meados do século XIX principalemnte na África e Estados Unidos.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B06W7KyzS</t>
+  </si>
+  <si>
+    <t>Amor e Ódio</t>
+  </si>
+  <si>
+    <t>A história se passa nas décadas de 1930 e 1940, abordando os períodos durante e após a Guerra Civil Espanhola e a Segunda Guerra Mundial. Trata-se de um drama envolvendo um triângulo amoroso, traições, crimes passionais e políticos, com personagens de personalidades ambíguas.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B05nNXv5D</t>
+  </si>
+  <si>
+    <t>A Vila</t>
+  </si>
+  <si>
+    <t>A Obra conta a historia de Athena, Andreas e de seus 4 filhos que vivem numa aldeia de pescadores de sardinhas na Grécia. O drama familiar se passa nas primeiras décadas do século XX explorando o amor, a paixão, as tragédias e a felicidade que permeou entre seus membros.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B00Abz1w9</t>
+  </si>
+  <si>
+    <t>Os Dois Irmãos</t>
+  </si>
+  <si>
+    <t>Neste livro, dois irmãos da região da Campagna, na Italia dos anos 1860, vivem uma bela historia de redenção e superação, denso e imprevisível como é a realidade da vida.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B099y4kAd</t>
+  </si>
+  <si>
+    <t>Esta obra contada pelos próprios personagens, nos da conta das dificuldades e tragédias, que uma família de classe média da Síria, passou durante a guerra civil naquele pais. Mas também mostra como eles se tornaram símbolos de resiliência e esperança diante das mais sombrias situações.</t>
+  </si>
+  <si>
+    <t>Os Refugiados </t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0g7NULvj</t>
+  </si>
+  <si>
+    <t>Destinos Cruzados: Parte 2</t>
+  </si>
+  <si>
+    <t>o jovem Willian que depois de se tornar um agente da Inteligencia Britanica - MI6, vai para Hong Kong dos anos 1960 em busca de sua mãe desaparecida.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0admSdvz</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B062ef4xG</t>
+  </si>
+  <si>
+    <t>O Reino</t>
+  </si>
+  <si>
+    <t>história de homens poderosos que desejam tudo, inclusive viver para sempre.</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B09rWOUcM</t>
+  </si>
+  <si>
+    <t>N°</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B09nhHaLT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -441,6 +668,32 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF0F1111"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFF6ECD9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -480,10 +733,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -491,14 +745,43 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -512,6 +795,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -809,20 +1096,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -1039,346 +1326,719 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="46" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" style="15"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="26.1796875" customWidth="1"/>
+    <col min="7" max="7" width="35.1796875" customWidth="1"/>
+    <col min="8" max="8" width="33.7265625" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.4">
+      <c r="B1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="4" spans="1:8" ht="28" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+    </row>
+    <row r="4" spans="1:10" ht="28" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="J4" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="50" x14ac:dyDescent="0.35">
+      <c r="A5" s="15">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="7" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="I5" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="J5" s="12"/>
+    </row>
+    <row r="6" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="15">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="7" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="I6" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="50" x14ac:dyDescent="0.35">
+      <c r="A7" s="15">
+        <v>3</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="7" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="I7" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="15">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="I8" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="15">
+        <v>5</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="7" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="I9" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="25" x14ac:dyDescent="0.35">
+      <c r="A10" s="15">
+        <v>6</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="7" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="I10" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J10" s="12"/>
+    </row>
+    <row r="11" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="15">
+        <v>7</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="7" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="I11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="15">
+        <v>8</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="7" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="I12" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="J12" s="12"/>
+    </row>
+    <row r="13" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="15">
+        <v>9</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="7" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="I13" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="J13" s="14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="15">
+        <v>10</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="7" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="I14" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="J14" s="14" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="15">
+        <v>11</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="7" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="25" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="I15" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="J15" s="14" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A16" s="15">
+        <v>12</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="7" t="s">
         <v>115</v>
       </c>
+      <c r="I16" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="15">
+        <v>13</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="15">
+        <v>14</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="15">
+        <v>15</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="J19" s="14" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="15">
+        <v>16</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="J20" s="14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="25" x14ac:dyDescent="0.35">
+      <c r="A21" s="15">
+        <v>17</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="15">
+        <v>18</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="15">
+        <v>19</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="15">
+        <v>20</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="15">
+        <v>21</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="I25" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="J25" s="14" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="15">
+        <v>22</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="15">
+        <v>23</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="J27" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="15">
+        <v>24</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="J28" s="14" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="15">
+        <v>25</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" s="15">
+        <v>26</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="J30" s="14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" s="15">
+        <v>27</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" s="15">
+        <v>28</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" s="15">
+        <v>29</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B34" s="7"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B35" s="7"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B36" s="7"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B37" s="7"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B38" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B1:G1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="I21" r:id="rId1" xr:uid="{3521BF82-1627-441E-B35F-749752FF56E1}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1393,10 +2053,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">

</xml_diff>